<commit_message>
ajustement avant new feature comparaison
</commit_message>
<xml_diff>
--- a/export/excel/rapport_chromebox_enterprise_g4_general.xlsx
+++ b/export/excel/rapport_chromebox_enterprise_g4_general.xlsx
@@ -16,11 +16,11 @@
     <sheet name="Périphériques" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPU'!$A$3:$D$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mémoire RAM'!$A$3:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stockage'!$A$3:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPU'!$A$3:$D$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mémoire RAM'!$A$3:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stockage'!$A$3:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Batterie'!$A$3:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Réseau'!$A$3:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Réseau'!$A$3:$F$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Périphériques'!$A$3:$E$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -592,7 +592,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>154.0.8037.96</t>
+          <t>154.0.8037.151</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -770,7 +770,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:30:41</t>
+          <t>2026-10-19 07:46:47</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -785,19 +785,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:29:40</t>
+          <t>2026-10-19 07:45:43</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:27:40</t>
+          <t>2026-10-19 07:43:43</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -836,12 +836,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:25:40</t>
+          <t>2026-10-19 07:41:43</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -858,12 +858,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:23:40</t>
+          <t>2026-10-19 07:39:43</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:21:40</t>
+          <t>2026-10-19 07:37:43</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -902,7 +902,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:19:40</t>
+          <t>2026-10-19 07:35:43</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:17:40</t>
+          <t>2026-10-19 07:33:43</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -946,7 +946,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:15:40</t>
+          <t>2026-10-19 07:31:43</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -968,12 +968,12 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:13:40</t>
+          <t>2026-10-19 07:29:43</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -990,12 +990,12 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:11:40</t>
+          <t>2026-10-19 07:27:43</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1012,7 +1012,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:30:40</t>
+          <t>2026-10-19 04:46:43</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1022,24 +1022,24 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Package id 0</t>
+          <t>Core 11</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>46</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:29:40</t>
+          <t>2026-10-19 04:45:43</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1056,7 +1056,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:08:39</t>
+          <t>2026-10-16 10:04:15</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1071,19 +1071,19 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>57</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:07:37</t>
+          <t>2026-10-16 10:03:15</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1100,29 +1100,29 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:05:37</t>
+          <t>2026-10-16 07:31:27</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Core 11</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>59</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:03:37</t>
+          <t>2026-10-16 07:30:26</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -1144,12 +1144,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:01:37</t>
+          <t>2026-10-16 07:28:26</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:59:37</t>
+          <t>2026-10-16 07:26:26</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1188,12 +1188,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:57:37</t>
+          <t>2026-10-16 07:24:26</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1210,12 +1210,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:55:37</t>
+          <t>2026-10-16 07:22:26</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1232,12 +1232,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:53:37</t>
+          <t>2026-10-16 07:20:26</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1254,12 +1254,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:51:37</t>
+          <t>2026-10-16 07:18:26</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1276,12 +1276,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:49:37</t>
+          <t>2026-10-16 07:16:26</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1298,34 +1298,34 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:08:38</t>
+          <t>2026-10-16 07:14:26</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Core 11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:07:37</t>
+          <t>2026-10-16 07:12:26</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1342,34 +1342,34 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:05:37</t>
+          <t>2026-10-16 04:31:26</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Core 4</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>38</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:03:37</t>
+          <t>2026-10-16 04:30:26</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:01:37</t>
+          <t>2026-10-15 13:31:59</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -1396,19 +1396,19 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Core 11</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>59</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:59:37</t>
+          <t>2026-10-15 13:30:56</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1430,7 +1430,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:57:37</t>
+          <t>2026-10-15 13:28:56</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1452,12 +1452,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:55:37</t>
+          <t>2026-10-15 13:26:56</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -1474,12 +1474,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:53:37</t>
+          <t>2026-10-15 13:24:56</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -1496,12 +1496,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:51:37</t>
+          <t>2026-10-15 13:22:56</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -1518,12 +1518,12 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:49:37</t>
+          <t>2026-10-15 13:20:56</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -1540,34 +1540,34 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:08:36</t>
+          <t>2026-10-15 13:18:56</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Package id 0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:07:36</t>
+          <t>2026-10-15 13:16:56</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -1584,34 +1584,34 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:06:32</t>
+          <t>2026-10-15 13:14:56</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Package id 0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:05:33</t>
+          <t>2026-10-15 13:12:56</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 04:42:14</t>
+          <t>2026-10-15 10:31:58</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -1638,24 +1638,24 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Core 4</t>
+          <t>Core 11</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>57</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 04:41:14</t>
+          <t>2026-10-15 10:30:56</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -1669,8 +1669,976 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:28:56</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:26:56</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:24:56</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:22:56</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:20:56</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:18:56</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:16:56</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:14:56</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:12:56</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:31:57</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Core 11</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30:55</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:28:55</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:26:55</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:24:55</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:22:55</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:20:55</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:18:55</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:16:55</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:14:55</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:12:55</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 04:31:55</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Package id 0</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 04:30:55</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:04:21</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Core 11</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:03:19</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:01:19</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:59:19</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:57:19</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:55:19</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:53:19</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:51:19</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:49:19</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:47:19</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:45:19</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:04:20</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Core 11</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:03:19</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:01:19</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:59:19</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:57:19</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:55:19</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:53:19</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:51:19</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:49:19</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:47:19</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:45:19</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:D45"/>
+  <autoFilter ref="A3:D89"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -1684,7 +2652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1737,12 +2705,12 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:30:43</t>
+          <t>2026-10-19 07:46:49</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>1012.73 Mo</t>
+          <t>762.97 Mo</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -1752,19 +2720,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>37986761</t>
+          <t>48383581</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:08:40</t>
+          <t>2026-10-19 04:46:47</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>480.65 Mo</t>
+          <t>5.28 Go</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1774,12 +2742,56 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>77650027</t>
+          <t>1479775</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16 10:04:16</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>5.56 Go</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>8.00 Go</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>67641189</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:31:28</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>945.62 Mo</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>8.00 Go</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>40803388</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D6"/>
+  <autoFilter ref="A3:D8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -1793,7 +2805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1846,7 +2858,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:30:43</t>
+          <t>2026-10-19 07:46:49</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1868,7 +2880,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:08:40</t>
+          <t>2026-10-19 04:46:47</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1887,8 +2899,52 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16 10:04:16</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>SSSTC CL4-3D256-HP</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>238.47 Go</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:31:28</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>SSSTC CL4-3D256-HP</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>238.47 Go</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:D6"/>
+  <autoFilter ref="A3:D8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -1983,7 +3039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2052,7 +3108,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 07:34:27</t>
+          <t>2026-10-19 04:47:38</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2084,7 +3140,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 06:34:27</t>
+          <t>2026-10-16 11:39:53</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -2116,7 +3172,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 05:34:27</t>
+          <t>2026-10-16 10:02:33</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2148,7 +3204,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:34:27</t>
+          <t>2026-10-16 09:32:33</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -2180,7 +3236,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:53:43</t>
+          <t>2026-10-16 08:32:33</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -2212,7 +3268,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 13:08:43</t>
+          <t>2026-10-16 07:32:33</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -2244,7 +3300,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 12:08:43</t>
+          <t>2026-10-16 06:32:33</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -2276,7 +3332,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 11:08:43</t>
+          <t>2026-10-16 05:32:33</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -2308,7 +3364,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 10:08:43</t>
+          <t>2026-10-16 04:32:33</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -2340,7 +3396,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 09:08:43</t>
+          <t>2026-10-15 13:48:32</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -2372,7 +3428,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 08:08:43</t>
+          <t>2026-10-15 13:33:32</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -2404,7 +3460,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:08:43</t>
+          <t>2026-10-15 12:33:32</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -2436,7 +3492,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 07:06:33</t>
+          <t>2026-10-15 11:33:32</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -2468,7 +3524,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 06:57:17</t>
+          <t>2026-10-15 10:33:32</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -2500,7 +3556,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 06:42:16</t>
+          <t>2026-10-15 09:33:32</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -2532,7 +3588,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 05:42:16</t>
+          <t>2026-10-15 08:33:32</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -2564,7 +3620,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-10-05 04:42:16</t>
+          <t>2026-10-15 07:33:32</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -2593,8 +3649,328 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 06:33:32</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 05:33:32</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 04:33:32</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:49:34</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:04:34</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:04:34</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:04:34</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:04:34</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:04:34</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:04:34</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.126</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>172.22.68.1</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>ETHERNET</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>1000000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F21"/>
+  <autoFilter ref="A3:F31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -2669,7 +4045,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:33:27</t>
+          <t>2026-10-19 04:46:39</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2696,7 +4072,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:33:27</t>
+          <t>2026-10-19 04:46:39</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -2723,7 +4099,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:33:27</t>
+          <t>2026-10-19 04:46:39</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2750,7 +4126,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:33:27</t>
+          <t>2026-10-19 04:46:39</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -2777,7 +4153,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-06 04:33:27</t>
+          <t>2026-10-19 04:46:39</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">

</xml_diff>